<commit_message>
Publish Base Profiles v2.0.0.
This publication was approved some time ago, but publishing failed with the IG publisher v. 2.0.17. Goes through now.
</commit_message>
<xml_diff>
--- a/fhir/finnish-base-profiles/CodeSystem-fi-base-release-for-patient-viewing-cs.xlsx
+++ b/fhir/finnish-base-profiles/CodeSystem-fi-base-release-for-patient-viewing-cs.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2.0.0-rc2</t>
+    <t>2.0.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -48,7 +48,7 @@
     <t>Status</t>
   </si>
   <si>
-    <t>draft</t>
+    <t>active</t>
   </si>
   <si>
     <t>Experimental</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-05-11T20:18:22+03:00</t>
+    <t>2025-10-05T18:45:07+03:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>